<commit_message>
docs: 老师跟踪表格回填 D5/D6 实测（#1/#2 Mathlib 落地、#30 lemma A/B、#31 leansearch 数据结论、#32 闭环、#33 基线）
</commit_message>
<xml_diff>
--- a/老师要求跟踪-资料库表格.xlsx
+++ b/老师要求跟踪-资料库表格.xlsx
@@ -619,12 +619,12 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>已完成(基线验证)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>代码有真实Lean编译验证，但验证路径(setup_lean.sh)显式设为单文件无mathlib；mathlib实际未接入，多数环境降级unknown。部分实现</t>
+          <t>已核实并打通：Mathlib.Tactic 依赖闭包实测 337 olean/0.11GB；deploy/mathlib-olean 已打包(110MB)并编译探针验证 norm_num/ring/linarith/nlinarith/positivity/omega 全可用。验证目录已挂载 LEAN_PATH，硬验证不再降级 unknown</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -661,12 +661,12 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>待办</t>
+          <t>已完成(方案A)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>未实现。验证路径无mathlib，mathlib工具链在磁盘但未接到验证编译目录，需先接入再AB测试</t>
+          <t>方案 A 可行：Mathlib 闭包仅 110MB（此前 1.5-3GB 估算错误，根因是按目录拷贝）。tools/package_mathlib.py 按依赖清单打包 + 自验通过，可随比赛包携带</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1837,12 +1837,12 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>待办</t>
+          <t>部分完成(A/B 已测)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>仅有单题内共享黑板；无 lemma 级记忆/复用（引理核验角色默认关闭）。待新增 lemma 记忆模块。</t>
+          <t>题目内 lemma 累积已真正接通（子目标结论写入 lemma_repo + 提示词注入，此前是无人写入的假钥匙）。45 题 A/B 实测：净 0.0pp（4 挽回 vs 4 真回退），数论子域 +23pp(31→54%)。保持默认关，按领域开启待后续</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -1879,12 +1879,12 @@
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>待办</t>
+          <t>已完成(数据结论)</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Mathlib 通道已打通(lean↔mathlib)；leansearch 定理检索尚未接入，待评估试用。</t>
+          <t>已实现并做 3 题 mini A/B：开=0 挽回、1 回退，耗时+19s/题。关键词打分器只对英文/mathlib 风格查询有效，中文/LaTeX 查询返回空。结论：保持关闭，升级语义检索(嵌入)为后续项</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -1921,12 +1921,12 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>待办</t>
+          <t>部分完成</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>已有 Lean 前置形式化(理解)与答案验证(检测)两端；"搜定理→informal推理→翻译Lean→审核"的闭环尚未打通。</t>
+          <t>闭环已具备：前置形式化(理解) → 骨架 Lean 语法审核 → 子目标求解 → 结构化 bug report 验证。验证-精炼循环依 IMO2025 论文落地（验证者≠解题者、问题二分、连续通过验收）</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>部分完成(A/B 已测)</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>lean↔mathlib 通道已搭建并修复 verify() 误判 bug；让 AI 主动用 Mathlib 解题尚在尝试。</t>
+          <t>lean↔mathlib 通道已通；DeepSeek 夜降成本方案待验证。45 题基线 22.2%，expr_wrong 占 69%（推理深度是主瓶颈，验证-精炼循环是主杠杆）</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">

</xml_diff>

<commit_message>
chore: run_phase0_eval override 支持 list/dict（preverify 按档位 A/B 用）+ debug15 排查题集
</commit_message>
<xml_diff>
--- a/老师要求跟踪-资料库表格.xlsx
+++ b/老师要求跟踪-资料库表格.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -171,6 +171,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -536,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1974,6 +1977,486 @@
       <c r="H34" s="3" t="inlineStr">
         <is>
           <t>李老师8/26 19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>持续推进测试基准实验，并明确当前存在哪些关键问题（阻塞项）。</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>测试基准</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>本地以 45 题为一轮，单轮 2-3 小时；比赛端由 lsq 同步优化，待其完成后再对齐修改。当前三个已知 bug：soft_budget 无人消费、lemma_repo 无人写入、leansearch 中文查询全空。</t>
+        </is>
+      </c>
+      <c r="H35" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/28 17:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>评估定理检索环节的开销与有效性；老师判断“大模型直接调用定理造成的时间开销较大”。</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>验证/Mathlib</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-28T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>已把简单题的 Lean 前置（帮助理解题目那一次）去掉，仅 deep 难题保留。leansearch 单次默认返回 5 条。实测一次调用链路：检索 7 条 → 去重去掉 4 条 → 剩 3 条有用 → 最终只用到 1 条，冗余高、转化率低。当前缺少定理调用埋点，无法量化调用频次与去重后定理数。</t>
+        </is>
+      </c>
+      <c r="H36" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/28 18:37 / 8/29 16:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>把 Mathlib 精简为“仅保留会用到的部分”，并随环境直接上传到比赛平台（比赛平台不带 Lean4/Mathlib）。</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>系统架构</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F37" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr">
+        <is>
+          <t>按依赖闭包裁剪：Mathlib.Tactic 实测 337 olean / 0.11GB（此前 1.5-3GB 系按目录统计的误判）。改为随包上传。待确认：比赛平台是否真的未预装 Lean4/Mathlib。</t>
+        </is>
+      </c>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 15:46-15:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="15" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>先考察本地环境下针对测试基准能做到的“理想正确率”上限，给出目标值。</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>测试基准</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F38" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr">
+        <is>
+          <t>IMO 类题目引入本套工具后 26% → 41%。修完全部已知 bug 预期稳定 40%+。比赛端因答案格式要求更严格，需先做格式适配再测。单轮实验成本 2-3 小时/45 题，是主要瓶颈。</t>
+        </is>
+      </c>
+      <c r="H38" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 16:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>统计题目没做对的原因：是 Lean 审核多次不通过，还是其它环节？给出归因分布。</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>测试基准</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>已完成(数据结论)</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>归因已明确：Lean 审核失败占少数（不通过会降级放行）；主因是时间分配错误——Lean 前置（形式化 LLM 调用 + 每次约 21s 的 mathlib 编译 + 骨架审核）叠加子目标规划耗尽时间预算，导致真正写题的预算不足。对策为提高整体时间预算。</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 16:15-16:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="15" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="15" t="inlineStr">
+        <is>
+          <t>对被调用的定理做记录（埋点），核实是否“调用次数频繁但调用的定理个数并不多”。</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>验证/Mathlib</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F40" s="15" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="G40" s="15" t="inlineStr">
+        <is>
+          <t>目前没有任何定理调用记录，需先补埋点（调用次数 / 命中数 / 去重后条数 / 最终被采用条数）再观察。</t>
+        </is>
+      </c>
+      <c r="H40" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 16:26-16:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>移除按题型分流的策略：IMO 基本全为证明题，题型分支反而拉低证明题正确率，应让 AI 按自身流程作答。</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>系统架构</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr">
+        <is>
+          <t>确认本地 IMO 题库全为证明题。解答题/证明题分流实测降低证明题正确率，计划移除该分支。老师补充：计算题同样含有证明成分，且主要依赖依赖链，不应把计算题排除在 Lean/定理检索之外。</t>
+        </is>
+      </c>
+      <c r="H41" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 23:07-23:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="15" t="inlineStr">
+        <is>
+          <t>明确单个子目标应检索出几条定理（top-k），并澄清“命中”的定义（命中不等于编译通过）。</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>验证/Mathlib</t>
+        </is>
+      </c>
+      <c r="D42" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F42" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="inlineStr">
+        <is>
+          <t>命中链路已澄清：先选相似候选 → 去重 → 验证 → 才是对 Lean 真正有用的。当前默认单次 5 条（上限）。实测 7 条→去重去掉 4 条→剩 3 条有用→最终用到 1 条。下一步在时间开销与返回条数间做权衡，并继续优化定理种类（已裁剪过一轮）。</t>
+        </is>
+      </c>
+      <c r="H42" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 23:13-23:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>参考《LeanSearch v2: Global Premise Retrieval for Lean 4 Theorem Proving》(arXiv:2605.13137v2) 改进定理检索。</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>验证/Mathlib</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F43" s="15" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="G43" s="15" t="inlineStr">
+        <is>
+          <t>论文已下载并入 ima 知识库「书生ai」。要点：双模式（standard 单查询 nDCG@10=0.62 + reasoning 的 sketch-retrieve-reflect 迭代循环）；MathlibMPR（69 题）下 10 候选内恢复 46.1% 真值前提组；接入固定 prover 后证明成功率 4%→20%。关键差异：我方 leansearch 仅在证明题启用，而老师指出计算题同样依赖定理依赖链。标准模式已开放 API（leansearch.net）。</t>
+        </is>
+      </c>
+      <c r="H43" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 23:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="15" t="inlineStr">
+        <is>
+          <t>解答中若用到某个定理，书生（推理模型）侧是否需要一并给出该定理的证明？</t>
+        </is>
+      </c>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>模型harness</t>
+        </is>
+      </c>
+      <c r="D44" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="G44" s="15" t="inlineStr">
+        <is>
+          <t>已答复老师：是需要的。需在提示词与输出格式中落实“引用定理须附带其证明/依据”。</t>
+        </is>
+      </c>
+      <c r="H44" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 23:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="15" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>保证时间充足、一步步做扎实：提高整体时间预算，与比赛的 6.5 小时上限对齐。</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>系统架构</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="F45" s="15" t="inlineStr">
+        <is>
+          <t>进行中</t>
+        </is>
+      </c>
+      <c r="G45" s="15" t="inlineStr">
+        <is>
+          <t>本地限定 5h，比赛限 6.5h。计划提高预算并重新校准各阶段配额（Lean 前置 / 子目标规划 / 写题）。老师要求不急于求成，逐步做扎实。</t>
+        </is>
+      </c>
+      <c r="H45" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 16:20-16:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>验证“增加候选数量的收益 &lt; 重复验证精炼的收益”这一结论，作为后续调优的方向约束。</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>测试基准</t>
+        </is>
+      </c>
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-29T00:00:00Z</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>已完成(数据结论)</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr">
+        <is>
+          <t>IMO 类题目 26%→41% 的过程中实测：堆候选数量收益小于重复验证精炼，与《Winning Gold at IMO 2025》证据一致（best-of-32 仅 31.6%，加验证精炼后 85.7%）。结论：任何“牺牲验证/协作轮数换取更多候选”的调优方向应予否决。</t>
+        </is>
+      </c>
+      <c r="H46" s="15" t="inlineStr">
+        <is>
+          <t>李老师8/29 16:06</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2510,7 @@
         </is>
       </c>
       <c r="B2" s="12">
-        <f>COUNTIF(老师要求跟踪!$F$2:$F$34,A2)</f>
+        <f>COUNTIF(老师要求跟踪!$F$2:$F$46,A2)</f>
         <v/>
       </c>
       <c r="C2" s="11" t="inlineStr">
@@ -2036,7 +2519,7 @@
         </is>
       </c>
       <c r="D2" s="12">
-        <f>COUNTIF(老师要求跟踪!$E$2:$E$34,C2)</f>
+        <f>COUNTIF(老师要求跟踪!$E$2:$E$46,C2)</f>
         <v/>
       </c>
     </row>
@@ -2047,7 +2530,7 @@
         </is>
       </c>
       <c r="B3" s="12">
-        <f>COUNTIF(老师要求跟踪!$F$2:$F$34,A3)</f>
+        <f>COUNTIF(老师要求跟踪!$F$2:$F$46,A3)</f>
         <v/>
       </c>
       <c r="C3" s="11" t="inlineStr">
@@ -2056,7 +2539,7 @@
         </is>
       </c>
       <c r="D3" s="12">
-        <f>COUNTIF(老师要求跟踪!$E$2:$E$34,C3)</f>
+        <f>COUNTIF(老师要求跟踪!$E$2:$E$46,C3)</f>
         <v/>
       </c>
     </row>
@@ -2067,7 +2550,7 @@
         </is>
       </c>
       <c r="B4" s="12">
-        <f>COUNTIF(老师要求跟踪!$F$2:$F$34,A4)</f>
+        <f>COUNTIF(老师要求跟踪!$F$2:$F$46,A4)</f>
         <v/>
       </c>
       <c r="C4" s="11" t="inlineStr">
@@ -2076,7 +2559,7 @@
         </is>
       </c>
       <c r="D4" s="12">
-        <f>COUNTIF(老师要求跟踪!$E$2:$E$34,C4)</f>
+        <f>COUNTIF(老师要求跟踪!$E$2:$E$46,C4)</f>
         <v/>
       </c>
     </row>
@@ -2100,6 +2583,7 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
@@ -2211,6 +2695,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>

</xml_diff>